<commit_message>
Restore intro video, handshake image, and fix horizontal scrolling
- Restore video files (intro.mp4, intro-mobile.mp4, intro.webm) from git history
- Restore IntroTransition component and CSS for intro animation
- Restore handshake image and logo assets
- Update App.jsx to include intro transition on homepage
- Restore original Home.jsx with handshake imagery
- Update assets manifest with all image references
- Fix horizontal scrolling by adding overflow-x:hidden to html/body
- Consolidate working files in zip folder, remove react-project duplicates

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/react-project/backend/data/contact-submissions.xlsx
+++ b/react-project/backend/data/contact-submissions.xlsx
@@ -31,19 +31,19 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Excel Test 15:33:49</t>
-  </si>
-  <si>
-    <t>excel@example.com</t>
-  </si>
-  <si>
-    <t>University / Institution partnership</t>
-  </si>
-  <si>
-    <t>Checking that submissions land in the Excel workbook.</t>
-  </si>
-  <si>
-    <t>mshoekdbuz4q3v</t>
+    <t>Sujaynithish N</t>
+  </si>
+  <si>
+    <t>sujaynithish2004@gmail.com</t>
+  </si>
+  <si>
+    <t>Students &amp; Graduates — launch my career</t>
+  </si>
+  <si>
+    <t>ji hi iam intersted</t>
+  </si>
+  <si>
+    <t>mshtmyth0a81fh</t>
   </si>
 </sst>
 </file>
@@ -466,7 +466,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>46240.648505543984</v>
+        <v>46240.75024228009</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>

</xml_diff>